<commit_message>
Remove legacy venue names from code paths and workbook metadata
</commit_message>
<xml_diff>
--- a/eval/ras_qa_nvidia_eval.xlsx
+++ b/eval/ras_qa_nvidia_eval.xlsx
@@ -4,9 +4,7 @@
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28730"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sktlg\OneDrive\바탕 화면\Neurips2025\"/>
-    </mc:Choice>
+    <mc:Choice Requires="x15"/>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A7F6AF1-EAF3-44DE-8A12-EAB2C16AA556}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>

</xml_diff>